<commit_message>
hide the previous weeks in the weekly scoring Excel workbook
</commit_message>
<xml_diff>
--- a/public/results/2026/2026 Weekly Stats - Week 2.xlsx
+++ b/public/results/2026/2026 Weekly Stats - Week 2.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D5C50D-05E3-B74E-AE3F-9C7CDB9C4C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFD3D2D-7DF2-4B5E-B988-17FB507B53F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44040" yWindow="2680" windowWidth="29860" windowHeight="16420" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1830" yWindow="15" windowWidth="18450" windowHeight="10785" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="14" r:id="rId1"/>
     <sheet name="Weekly Stats" sheetId="11" r:id="rId2"/>
     <sheet name="Point System" sheetId="7" r:id="rId3"/>
-    <sheet name="Week 1" sheetId="4" r:id="rId4"/>
+    <sheet name="Week 1" sheetId="4" state="hidden" r:id="rId4"/>
     <sheet name="Week 2" sheetId="15" r:id="rId5"/>
   </sheets>
   <externalReferences>
@@ -330,7 +330,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1242,7 +1242,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1506,97 +1506,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1606,17 +1522,98 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1640,117 +1637,13 @@
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
+      <xxl21:relativeUrl r:id="rId2"/>
     </xxl21:alternateUrls>
     <sheetNames>
-      <sheetName val="Instructions"/>
       <sheetName val="Point System"/>
-      <sheetName val="18-hole scores"/>
-      <sheetName val="9-hole scores"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="A4">
-            <v>-5</v>
-          </cell>
-          <cell r="B4">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>-4</v>
-          </cell>
-          <cell r="B5">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>-3</v>
-          </cell>
-          <cell r="B6">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>-2</v>
-          </cell>
-          <cell r="B7">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>-1</v>
-          </cell>
-          <cell r="B8">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>0</v>
-          </cell>
-          <cell r="B9">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>1</v>
-          </cell>
-          <cell r="B10">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>2</v>
-          </cell>
-          <cell r="B11">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>3</v>
-          </cell>
-          <cell r="B12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>4</v>
-          </cell>
-          <cell r="B13">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>5</v>
-          </cell>
-          <cell r="B14">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>6</v>
-          </cell>
-          <cell r="B15">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="0" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2074,42 +1967,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75685173-5684-4D7E-8458-1B841D06EDCF}">
   <dimension ref="A1:Z21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="14.140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="23" style="3" customWidth="1"/>
     <col min="2" max="2" width="15" style="3" customWidth="1"/>
     <col min="3" max="11" width="5" style="3" customWidth="1"/>
-    <col min="12" max="12" width="5.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.1640625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="7.5" style="3" customWidth="1"/>
-    <col min="15" max="15" width="17.1640625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="8.6640625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="15.1640625" style="3" customWidth="1"/>
-    <col min="18" max="18" width="13.6640625" style="3" customWidth="1"/>
-    <col min="19" max="19" width="8.6640625" style="3" customWidth="1"/>
-    <col min="20" max="20" width="8.6640625" style="33" customWidth="1"/>
-    <col min="21" max="26" width="8.6640625" style="3" customWidth="1"/>
-    <col min="27" max="16384" width="14.1640625" style="3"/>
+    <col min="12" max="12" width="5.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.140625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="7.42578125" style="3" customWidth="1"/>
+    <col min="15" max="15" width="17.140625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" style="3" customWidth="1"/>
+    <col min="17" max="17" width="15.140625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="3" customWidth="1"/>
+    <col min="19" max="19" width="8.7109375" style="3" customWidth="1"/>
+    <col min="20" max="20" width="8.7109375" style="33" customWidth="1"/>
+    <col min="21" max="26" width="8.7109375" style="3" customWidth="1"/>
+    <col min="27" max="16384" width="14.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+    <row r="1" spans="1:26" ht="26.25">
+      <c r="A1" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
-      <c r="F1" s="133"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="133"/>
-      <c r="I1" s="133"/>
-      <c r="J1" s="133"/>
-      <c r="K1" s="133"/>
-      <c r="L1" s="133"/>
-      <c r="M1" s="133"/>
-      <c r="N1" s="133"/>
-      <c r="O1" s="133"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -2122,24 +2015,24 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A2" s="134" t="s">
+    <row r="2" spans="1:26">
+      <c r="A2" s="106" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="133"/>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="133"/>
-      <c r="K2" s="133"/>
-      <c r="L2" s="133"/>
-      <c r="M2" s="133"/>
-      <c r="N2" s="133"/>
-      <c r="O2" s="133"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -2152,7 +2045,7 @@
       <c r="Y2" s="2"/>
       <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" ht="19.5" thickBot="1">
       <c r="A3" s="4"/>
       <c r="B3" s="2"/>
       <c r="C3" s="5"/>
@@ -2180,7 +2073,7 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="18.75">
       <c r="A4" s="20" t="s">
         <v>16</v>
       </c>
@@ -2240,7 +2133,7 @@
       <c r="Y4" s="4"/>
       <c r="Z4" s="4"/>
     </row>
-    <row r="5" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="18.75">
       <c r="A5" s="23"/>
       <c r="B5" s="7" t="s">
         <v>22</v>
@@ -2293,7 +2186,7 @@
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
     </row>
-    <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="19.5" thickBot="1">
       <c r="A6" s="25"/>
       <c r="B6" s="26" t="s">
         <v>33</v>
@@ -2341,7 +2234,7 @@
       <c r="Y6" s="4"/>
       <c r="Z6" s="4"/>
     </row>
-    <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="18.75">
       <c r="A7" s="12"/>
       <c r="B7" s="13" t="s">
         <v>32</v>
@@ -2377,7 +2270,7 @@
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="19.5" thickBot="1">
       <c r="A8" s="16"/>
       <c r="B8" s="17" t="s">
         <v>34</v>
@@ -2439,7 +2332,7 @@
       <c r="X8" s="2"/>
       <c r="Z8" s="36"/>
     </row>
-    <row r="9" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="18.75">
       <c r="A9" s="12"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
@@ -2466,7 +2359,7 @@
       <c r="R9" s="31"/>
       <c r="T9" s="3"/>
     </row>
-    <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="19.5" thickBot="1">
       <c r="A10" s="16"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17" t="str">
@@ -2520,7 +2413,7 @@
       <c r="R10" s="31"/>
       <c r="T10" s="3"/>
     </row>
-    <row r="11" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="18.75">
       <c r="A11" s="12"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -2548,7 +2441,7 @@
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="19.5" thickBot="1">
       <c r="A12" s="16"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17" t="str">
@@ -2603,7 +2496,7 @@
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="18.75">
       <c r="A13" s="12"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2631,7 +2524,7 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="19.5" thickBot="1">
       <c r="A14" s="16"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17" t="str">
@@ -2686,7 +2579,7 @@
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="18.75">
       <c r="A15" s="12"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -2717,7 +2610,7 @@
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
     </row>
-    <row r="16" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="19.5" thickBot="1">
       <c r="A16" s="16"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17" t="str">
@@ -2775,7 +2668,7 @@
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
     </row>
-    <row r="17" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26" ht="18.75">
       <c r="A17" s="12"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -2806,7 +2699,7 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="19.5" thickBot="1">
       <c r="A18" s="16"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17" t="str">
@@ -2864,7 +2757,7 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26" ht="18.75">
       <c r="A19" s="12"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -2891,7 +2784,7 @@
       <c r="R19" s="31"/>
       <c r="T19" s="3"/>
     </row>
-    <row r="20" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="19.5" thickBot="1">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17" t="str">
@@ -2945,7 +2838,7 @@
       <c r="R20" s="31"/>
       <c r="T20" s="3"/>
     </row>
-    <row r="21" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:26" ht="15" customHeight="1">
       <c r="E21" s="30"/>
       <c r="G21" s="30"/>
       <c r="H21" s="30"/>
@@ -2968,117 +2861,117 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1EE897-404D-4ADC-856A-1E864FE4E3AA}">
   <dimension ref="A1:P30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="11.5" customWidth="1"/>
-    <col min="3" max="3" width="9.5" customWidth="1"/>
-    <col min="4" max="5" width="7.5" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" customWidth="1"/>
-    <col min="7" max="7" width="9.1640625" customWidth="1"/>
-    <col min="8" max="8" width="6.5" customWidth="1"/>
-    <col min="9" max="9" width="6.33203125" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" customWidth="1"/>
-    <col min="12" max="12" width="8.5" hidden="1" customWidth="1"/>
-    <col min="13" max="14" width="6.83203125" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="8.5" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="10.6640625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" customWidth="1"/>
+    <col min="4" max="5" width="7.42578125" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="6.42578125" customWidth="1"/>
+    <col min="9" max="9" width="6.28515625" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" hidden="1" customWidth="1"/>
+    <col min="13" max="14" width="6.85546875" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="8.42578125" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="10.7109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+    <row r="1" spans="1:16" s="1" customFormat="1" ht="24.95" customHeight="1" thickBot="1">
+      <c r="A1" s="114" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="130" t="s">
+      <c r="B1" s="115"/>
+      <c r="C1" s="120" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="120" t="s">
+      <c r="D1" s="110" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="121"/>
-      <c r="F1" s="117" t="s">
+      <c r="E1" s="111"/>
+      <c r="F1" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="127" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="102"/>
-      <c r="I1" s="102"/>
-      <c r="J1" s="102"/>
-      <c r="K1" s="103"/>
-      <c r="L1" s="112" t="s">
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="129"/>
+      <c r="L1" s="122" t="s">
         <v>43</v>
       </c>
-      <c r="M1" s="113"/>
-      <c r="N1" s="113"/>
-      <c r="O1" s="113"/>
-      <c r="P1" s="114"/>
-    </row>
-    <row r="2" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="126"/>
-      <c r="B2" s="127"/>
-      <c r="C2" s="131"/>
-      <c r="D2" s="122">
+      <c r="M1" s="123"/>
+      <c r="N1" s="123"/>
+      <c r="O1" s="123"/>
+      <c r="P1" s="124"/>
+    </row>
+    <row r="2" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A2" s="116"/>
+      <c r="B2" s="117"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="112">
         <v>46146</v>
       </c>
-      <c r="E2" s="123"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="104" t="s">
+      <c r="E2" s="113"/>
+      <c r="F2" s="108"/>
+      <c r="G2" s="130" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="106" t="s">
+      <c r="H2" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="110" t="s">
+      <c r="I2" s="136" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="104" t="s">
+      <c r="J2" s="130" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="108" t="s">
+      <c r="K2" s="134" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="115" t="s">
+      <c r="L2" s="125" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="115" t="s">
+      <c r="M2" s="125" t="s">
         <v>41</v>
       </c>
-      <c r="N2" s="115" t="s">
+      <c r="N2" s="125" t="s">
         <v>73</v>
       </c>
-      <c r="O2" s="115" t="s">
+      <c r="O2" s="125" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="115" t="s">
+      <c r="P2" s="125" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="128"/>
-      <c r="B3" s="129"/>
-      <c r="C3" s="131"/>
+    <row r="3" spans="1:16" s="1" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A3" s="118"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="121"/>
       <c r="D3" s="37" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="119"/>
-      <c r="G3" s="105"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="105"/>
-      <c r="K3" s="109"/>
-      <c r="L3" s="116"/>
-      <c r="M3" s="116"/>
-      <c r="N3" s="116"/>
-      <c r="O3" s="116"/>
-      <c r="P3" s="116"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F3" s="109"/>
+      <c r="G3" s="131"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="137"/>
+      <c r="J3" s="131"/>
+      <c r="K3" s="135"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="126"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="126"/>
+    </row>
+    <row r="4" spans="1:16" ht="15" customHeight="1">
       <c r="A4" s="38" t="s">
         <v>88</v>
       </c>
@@ -3117,7 +3010,7 @@
       <c r="O4" s="57"/>
       <c r="P4" s="64"/>
     </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="15" customHeight="1">
       <c r="A5" s="41" t="s">
         <v>52</v>
       </c>
@@ -3160,7 +3053,7 @@
       <c r="O5" s="59"/>
       <c r="P5" s="65"/>
     </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="15" customHeight="1">
       <c r="A6" s="41" t="s">
         <v>0</v>
       </c>
@@ -3201,7 +3094,7 @@
       <c r="O6" s="59"/>
       <c r="P6" s="65"/>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="15" customHeight="1">
       <c r="A7" s="41" t="s">
         <v>2</v>
       </c>
@@ -3242,7 +3135,7 @@
       <c r="O7" s="59"/>
       <c r="P7" s="65"/>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="15" customHeight="1">
       <c r="A8" s="41" t="s">
         <v>64</v>
       </c>
@@ -3281,7 +3174,7 @@
       <c r="O8" s="59"/>
       <c r="P8" s="65"/>
     </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="15" customHeight="1">
       <c r="A9" s="41" t="s">
         <v>49</v>
       </c>
@@ -3320,7 +3213,7 @@
       <c r="O9" s="59"/>
       <c r="P9" s="65"/>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="15" customHeight="1">
       <c r="A10" s="41" t="s">
         <v>47</v>
       </c>
@@ -3359,7 +3252,7 @@
       <c r="O10" s="59"/>
       <c r="P10" s="65"/>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="15" customHeight="1">
       <c r="A11" s="41" t="s">
         <v>68</v>
       </c>
@@ -3398,7 +3291,7 @@
       <c r="O11" s="59"/>
       <c r="P11" s="65"/>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="15" customHeight="1">
       <c r="A12" s="41" t="s">
         <v>81</v>
       </c>
@@ -3432,7 +3325,7 @@
       <c r="O12" s="59"/>
       <c r="P12" s="65"/>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="15" customHeight="1">
       <c r="A13" s="41" t="s">
         <v>0</v>
       </c>
@@ -3466,7 +3359,7 @@
       <c r="O13" s="59"/>
       <c r="P13" s="65"/>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="15" customHeight="1">
       <c r="A14" s="41" t="s">
         <v>83</v>
       </c>
@@ -3500,7 +3393,7 @@
       <c r="O14" s="59"/>
       <c r="P14" s="65"/>
     </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="15" customHeight="1">
       <c r="A15" s="41" t="s">
         <v>86</v>
       </c>
@@ -3534,7 +3427,7 @@
       <c r="O15" s="59"/>
       <c r="P15" s="65"/>
     </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="15" customHeight="1">
       <c r="A16" s="41" t="s">
         <v>56</v>
       </c>
@@ -3561,7 +3454,7 @@
       <c r="O16" s="59"/>
       <c r="P16" s="65"/>
     </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="15" customHeight="1">
       <c r="A17" s="41" t="s">
         <v>66</v>
       </c>
@@ -3588,7 +3481,7 @@
       <c r="O17" s="59"/>
       <c r="P17" s="65"/>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="15" customHeight="1">
       <c r="A18" s="41" t="s">
         <v>54</v>
       </c>
@@ -3615,7 +3508,7 @@
       <c r="O18" s="59"/>
       <c r="P18" s="65"/>
     </row>
-    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="15" customHeight="1">
       <c r="A19" s="41" t="s">
         <v>49</v>
       </c>
@@ -3642,7 +3535,7 @@
       <c r="O19" s="59"/>
       <c r="P19" s="65"/>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="15" customHeight="1">
       <c r="A20" s="41" t="s">
         <v>70</v>
       </c>
@@ -3669,7 +3562,7 @@
       <c r="O20" s="59"/>
       <c r="P20" s="65"/>
     </row>
-    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="15" customHeight="1">
       <c r="A21" s="41" t="s">
         <v>62</v>
       </c>
@@ -3696,7 +3589,7 @@
       <c r="O21" s="59"/>
       <c r="P21" s="65"/>
     </row>
-    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="15" customHeight="1">
       <c r="A22" s="41" t="s">
         <v>3</v>
       </c>
@@ -3723,7 +3616,7 @@
       <c r="O22" s="59"/>
       <c r="P22" s="65"/>
     </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="15" customHeight="1">
       <c r="A23" s="41" t="s">
         <v>60</v>
       </c>
@@ -3752,7 +3645,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="15" customHeight="1">
       <c r="A24" s="41" t="s">
         <v>54</v>
       </c>
@@ -3779,7 +3672,7 @@
       <c r="O24" s="59"/>
       <c r="P24" s="65"/>
     </row>
-    <row r="25" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="15" customHeight="1" thickBot="1">
       <c r="A25" s="72" t="s">
         <v>58</v>
       </c>
@@ -3806,7 +3699,7 @@
       <c r="O25" s="60"/>
       <c r="P25" s="66"/>
     </row>
-    <row r="26" spans="1:16" s="52" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" s="52" customFormat="1" ht="15.75" thickBot="1">
       <c r="A26" s="70"/>
       <c r="B26" s="69"/>
       <c r="C26" s="69"/>
@@ -3817,7 +3710,7 @@
       <c r="E26" s="68"/>
       <c r="F26" s="66"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16">
       <c r="C27" s="49"/>
       <c r="F27" s="50"/>
       <c r="G27" s="50"/>
@@ -3826,7 +3719,7 @@
       <c r="J27" s="50"/>
       <c r="K27" s="51"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16">
       <c r="C28" s="47" t="s">
         <v>6</v>
       </c>
@@ -3834,7 +3727,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16">
       <c r="C29" s="47" t="s">
         <v>7</v>
       </c>
@@ -3843,7 +3736,7 @@
       </c>
       <c r="F29" s="67"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16">
       <c r="C30" s="47" t="s">
         <v>38</v>
       </c>
@@ -3860,23 +3753,23 @@
     <sortCondition ref="A4:A25"/>
   </sortState>
   <mergeCells count="17">
-    <mergeCell ref="F1:F3"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="I2:I3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="O2:O3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="N2:N3"/>
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="F1:F3"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:C3"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3890,20 +3783,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E789909-84FC-488D-8D94-3FAD76B00BC6}">
   <dimension ref="A1:B1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" style="3" customWidth="1"/>
-    <col min="3" max="26" width="7.6640625" style="3" customWidth="1"/>
-    <col min="27" max="16384" width="12.6640625" style="3"/>
+    <col min="1" max="1" width="20.28515625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" style="3" customWidth="1"/>
+    <col min="3" max="26" width="7.7109375" style="3" customWidth="1"/>
+    <col min="27" max="16384" width="12.7109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" s="9" t="s">
         <v>27</v>
       </c>
@@ -3911,7 +3804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" s="10">
         <v>-5</v>
       </c>
@@ -3919,7 +3812,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2">
       <c r="A5" s="10">
         <v>-4</v>
       </c>
@@ -3927,7 +3820,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2">
       <c r="A6" s="10">
         <v>-3</v>
       </c>
@@ -3935,7 +3828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2">
       <c r="A7" s="10">
         <v>-2</v>
       </c>
@@ -3943,7 +3836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2">
       <c r="A8" s="10">
         <v>-1</v>
       </c>
@@ -3951,7 +3844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9" s="10">
         <v>0</v>
       </c>
@@ -3959,7 +3852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10" s="10">
         <v>1</v>
       </c>
@@ -3967,7 +3860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11" s="10">
         <v>2</v>
       </c>
@@ -3975,7 +3868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12" s="10">
         <v>3</v>
       </c>
@@ -3983,7 +3876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" s="10">
         <v>4</v>
       </c>
@@ -3991,7 +3884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2">
       <c r="A14" s="10">
         <v>5</v>
       </c>
@@ -3999,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2">
       <c r="A15" s="10">
         <v>6</v>
       </c>
@@ -4007,996 +3900,996 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1">
       <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:1" ht="14.25">
       <c r="A18" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="27" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="28" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="29" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="30" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="31" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="36" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="37" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="39" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="46" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="47" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="21" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:1" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
+    <row r="38" ht="15.75" customHeight="1"/>
+    <row r="39" ht="15.75" customHeight="1"/>
+    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1"/>
+    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A18" r:id="rId1" xr:uid="{BB8AB8C5-9F96-41D8-B252-ACC21DAB1BB3}"/>
@@ -5009,37 +4902,37 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{299C7D47-E383-421C-AFFB-D42B2CA94D59}">
   <dimension ref="A1:Z30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="14.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="11" width="5" style="3" customWidth="1"/>
-    <col min="12" max="12" width="5.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="5" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="26" width="8.6640625" style="3" customWidth="1"/>
-    <col min="27" max="16384" width="14.1640625" style="3"/>
+    <col min="15" max="15" width="14.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="26" width="8.7109375" style="3" customWidth="1"/>
+    <col min="27" max="16384" width="14.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+    <row r="1" spans="1:26" ht="26.25">
+      <c r="A1" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
-      <c r="F1" s="133"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="133"/>
-      <c r="I1" s="133"/>
-      <c r="J1" s="133"/>
-      <c r="K1" s="133"/>
-      <c r="L1" s="133"/>
-      <c r="M1" s="133"/>
-      <c r="N1" s="133"/>
-      <c r="O1" s="133"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -5052,24 +4945,24 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
-    <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="134" t="s">
+    <row r="2" spans="1:26" ht="15">
+      <c r="A2" s="106" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="133"/>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="133"/>
-      <c r="K2" s="133"/>
-      <c r="L2" s="133"/>
-      <c r="M2" s="133"/>
-      <c r="N2" s="133"/>
-      <c r="O2" s="133"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -5082,7 +4975,7 @@
       <c r="Y2" s="2"/>
       <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" ht="19.5" thickBot="1">
       <c r="A3" s="4"/>
       <c r="B3" s="2"/>
       <c r="C3" s="5"/>
@@ -5110,7 +5003,7 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="18.75">
       <c r="A4" s="20" t="s">
         <v>16</v>
       </c>
@@ -5168,7 +5061,7 @@
       <c r="Y4" s="4"/>
       <c r="Z4" s="4"/>
     </row>
-    <row r="5" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="18.75">
       <c r="A5" s="23"/>
       <c r="B5" s="7" t="s">
         <v>22</v>
@@ -5219,7 +5112,7 @@
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
     </row>
-    <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="19.5" thickBot="1">
       <c r="A6" s="25"/>
       <c r="B6" s="26" t="s">
         <v>33</v>
@@ -5267,7 +5160,7 @@
       <c r="Y6" s="4"/>
       <c r="Z6" s="4"/>
     </row>
-    <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="18.75">
       <c r="A7" s="12" t="s">
         <v>40</v>
       </c>
@@ -5325,7 +5218,7 @@
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="19.5" thickBot="1">
       <c r="A8" s="16"/>
       <c r="B8" s="17" t="s">
         <v>34</v>
@@ -5388,7 +5281,7 @@
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
     </row>
-    <row r="9" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="18.75">
       <c r="A9" s="12" t="s">
         <v>24</v>
       </c>
@@ -5444,7 +5337,7 @@
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
     </row>
-    <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="19.5" thickBot="1">
       <c r="A10" s="16"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17">
@@ -5505,7 +5398,7 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="18.75">
       <c r="A11" s="12" t="s">
         <v>80</v>
       </c>
@@ -5558,7 +5451,7 @@
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="19.5" thickBot="1">
       <c r="A12" s="16"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -5592,7 +5485,7 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="18.75">
       <c r="A13" s="12" t="s">
         <v>75</v>
       </c>
@@ -5645,7 +5538,7 @@
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="19.5" thickBot="1">
       <c r="A14" s="16"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -5679,7 +5572,7 @@
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="18.75">
       <c r="A15" s="12" t="s">
         <v>31</v>
       </c>
@@ -5735,7 +5628,7 @@
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
     </row>
-    <row r="16" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="19.5" thickBot="1">
       <c r="A16" s="16"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17">
@@ -5796,7 +5689,7 @@
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
     </row>
-    <row r="17" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26" ht="18.75">
       <c r="A17" s="12" t="s">
         <v>25</v>
       </c>
@@ -5852,7 +5745,7 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="19.5" thickBot="1">
       <c r="A18" s="16"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17">
@@ -5913,7 +5806,7 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26" ht="18.75">
       <c r="A19" s="12" t="s">
         <v>76</v>
       </c>
@@ -5969,7 +5862,7 @@
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="19.5" thickBot="1">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17">
@@ -6030,7 +5923,7 @@
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
     </row>
-    <row r="21" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26" ht="18.75">
       <c r="A21" s="12" t="s">
         <v>44</v>
       </c>
@@ -6086,7 +5979,7 @@
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
     </row>
-    <row r="22" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="19.5" thickBot="1">
       <c r="A22" s="16"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17">
@@ -6147,7 +6040,7 @@
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
     </row>
-    <row r="23" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:26" ht="18.75">
       <c r="A23" s="12" t="s">
         <v>77</v>
       </c>
@@ -6200,7 +6093,7 @@
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
     </row>
-    <row r="24" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="19.5" thickBot="1">
       <c r="A24" s="16"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -6234,7 +6127,7 @@
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
     </row>
-    <row r="25" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26" ht="18.75">
       <c r="A25" s="12" t="s">
         <v>23</v>
       </c>
@@ -6290,7 +6183,7 @@
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
     </row>
-    <row r="26" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="19.5" thickBot="1">
       <c r="A26" s="16"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17">
@@ -6351,7 +6244,7 @@
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
     </row>
-    <row r="27" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:26" ht="18.75">
       <c r="A27" s="12" t="s">
         <v>78</v>
       </c>
@@ -6404,7 +6297,7 @@
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
     </row>
-    <row r="28" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="19.5" thickBot="1">
       <c r="A28" s="16"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -6435,7 +6328,7 @@
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
     </row>
-    <row r="29" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26" ht="18.75">
       <c r="A29" s="12" t="s">
         <v>79</v>
       </c>
@@ -6491,7 +6384,7 @@
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
     </row>
-    <row r="30" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" ht="19.5" thickBot="1">
       <c r="A30" s="16"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17">
@@ -6568,37 +6461,37 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4934D7F3-41CA-D943-8BF9-D91C155D4533}">
   <dimension ref="A1:Z34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.1640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="14.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="11" width="5" style="3" customWidth="1"/>
-    <col min="12" max="12" width="5.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="5" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="26" width="8.6640625" style="3" customWidth="1"/>
-    <col min="27" max="16384" width="14.1640625" style="3"/>
+    <col min="15" max="15" width="14.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="26" width="8.7109375" style="3" customWidth="1"/>
+    <col min="27" max="16384" width="14.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+    <row r="1" spans="1:26" ht="26.25">
+      <c r="A1" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
-      <c r="F1" s="133"/>
-      <c r="G1" s="133"/>
-      <c r="H1" s="133"/>
-      <c r="I1" s="133"/>
-      <c r="J1" s="133"/>
-      <c r="K1" s="133"/>
-      <c r="L1" s="133"/>
-      <c r="M1" s="133"/>
-      <c r="N1" s="133"/>
-      <c r="O1" s="133"/>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="105"/>
+      <c r="L1" s="105"/>
+      <c r="M1" s="105"/>
+      <c r="N1" s="105"/>
+      <c r="O1" s="105"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -6611,24 +6504,24 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
-    <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="134" t="s">
+    <row r="2" spans="1:26" ht="15">
+      <c r="A2" s="106" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="133"/>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="133"/>
-      <c r="J2" s="133"/>
-      <c r="K2" s="133"/>
-      <c r="L2" s="133"/>
-      <c r="M2" s="133"/>
-      <c r="N2" s="133"/>
-      <c r="O2" s="133"/>
+      <c r="B2" s="105"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="105"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -6641,7 +6534,7 @@
       <c r="Y2" s="2"/>
       <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" ht="19.5" thickBot="1">
       <c r="A3" s="4"/>
       <c r="B3" s="2"/>
       <c r="C3" s="5"/>
@@ -6669,7 +6562,7 @@
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" ht="18.75">
       <c r="A4" s="20" t="s">
         <v>16</v>
       </c>
@@ -6727,7 +6620,7 @@
       <c r="Y4" s="4"/>
       <c r="Z4" s="4"/>
     </row>
-    <row r="5" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" ht="18.75">
       <c r="A5" s="23"/>
       <c r="B5" s="7" t="s">
         <v>22</v>
@@ -6778,7 +6671,7 @@
       <c r="Y5" s="4"/>
       <c r="Z5" s="4"/>
     </row>
-    <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="19.5" thickBot="1">
       <c r="A6" s="25"/>
       <c r="B6" s="26" t="s">
         <v>33</v>
@@ -6826,7 +6719,7 @@
       <c r="Y6" s="4"/>
       <c r="Z6" s="4"/>
     </row>
-    <row r="7" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" ht="18.75">
       <c r="A7" s="12" t="s">
         <v>77</v>
       </c>
@@ -6882,7 +6775,7 @@
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="19.5" thickBot="1">
       <c r="A8" s="16"/>
       <c r="B8" s="17" t="s">
         <v>34</v>
@@ -6945,7 +6838,7 @@
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
     </row>
-    <row r="9" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" ht="18.75">
       <c r="A9" s="12" t="s">
         <v>25</v>
       </c>
@@ -7001,7 +6894,7 @@
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
     </row>
-    <row r="10" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="19.5" thickBot="1">
       <c r="A10" s="16"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17">
@@ -7062,7 +6955,7 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" ht="18.75">
       <c r="A11" s="12" t="s">
         <v>31</v>
       </c>
@@ -7118,7 +7011,7 @@
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="19.5" thickBot="1">
       <c r="A12" s="16"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17">
@@ -7179,7 +7072,7 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" ht="18.75">
       <c r="A13" s="12" t="s">
         <v>90</v>
       </c>
@@ -7232,7 +7125,7 @@
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="19.5" thickBot="1">
       <c r="A14" s="16"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -7266,7 +7159,7 @@
       <c r="Y14" s="2"/>
       <c r="Z14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" ht="18.75">
       <c r="A15" s="12" t="s">
         <v>76</v>
       </c>
@@ -7274,7 +7167,7 @@
       <c r="C15" s="13">
         <v>4</v>
       </c>
-      <c r="D15" s="137">
+      <c r="D15" s="102">
         <v>3</v>
       </c>
       <c r="E15" s="13">
@@ -7295,7 +7188,7 @@
       <c r="J15" s="13">
         <v>4</v>
       </c>
-      <c r="K15" s="138">
+      <c r="K15" s="103">
         <v>4</v>
       </c>
       <c r="L15" s="14">
@@ -7322,7 +7215,7 @@
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
     </row>
-    <row r="16" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="19.5" thickBot="1">
       <c r="A16" s="16"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17">
@@ -7383,36 +7276,36 @@
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
     </row>
-    <row r="17" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26" ht="18.75">
       <c r="A17" s="12" t="s">
         <v>44</v>
       </c>
       <c r="B17" s="13"/>
-      <c r="C17" s="136">
-        <v>4</v>
-      </c>
-      <c r="D17" s="138">
-        <v>4</v>
-      </c>
-      <c r="E17" s="136">
-        <v>5</v>
-      </c>
-      <c r="F17" s="138">
+      <c r="C17" s="13">
+        <v>4</v>
+      </c>
+      <c r="D17" s="103">
+        <v>4</v>
+      </c>
+      <c r="E17" s="13">
+        <v>5</v>
+      </c>
+      <c r="F17" s="103">
         <v>2</v>
       </c>
-      <c r="G17" s="136">
-        <v>5</v>
-      </c>
-      <c r="H17" s="136">
+      <c r="G17" s="13">
+        <v>5</v>
+      </c>
+      <c r="H17" s="13">
         <v>6</v>
       </c>
-      <c r="I17" s="135">
-        <v>4</v>
-      </c>
-      <c r="J17" s="136">
-        <v>5</v>
-      </c>
-      <c r="K17" s="136">
+      <c r="I17" s="101">
+        <v>4</v>
+      </c>
+      <c r="J17" s="13">
+        <v>5</v>
+      </c>
+      <c r="K17" s="13">
         <v>5</v>
       </c>
       <c r="L17" s="14">
@@ -7439,7 +7332,7 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="19.5" thickBot="1">
       <c r="A18" s="16"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17">
@@ -7500,7 +7393,7 @@
       <c r="Y18" s="2"/>
       <c r="Z18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26" ht="18.75">
       <c r="A19" s="12" t="s">
         <v>91</v>
       </c>
@@ -7508,7 +7401,7 @@
       <c r="C19" s="13">
         <v>4</v>
       </c>
-      <c r="D19" s="138">
+      <c r="D19" s="103">
         <v>4</v>
       </c>
       <c r="E19" s="13">
@@ -7526,7 +7419,7 @@
       <c r="I19" s="13">
         <v>4</v>
       </c>
-      <c r="J19" s="138">
+      <c r="J19" s="103">
         <v>3</v>
       </c>
       <c r="K19" s="13">
@@ -7553,7 +7446,7 @@
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="19.5" thickBot="1">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -7587,12 +7480,12 @@
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
     </row>
-    <row r="21" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26" ht="18.75">
       <c r="A21" s="12" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="13"/>
-      <c r="C21" s="138">
+      <c r="C21" s="103">
         <v>3</v>
       </c>
       <c r="D21" s="13">
@@ -7643,7 +7536,7 @@
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
     </row>
-    <row r="22" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="19.5" thickBot="1">
       <c r="A22" s="16"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17">
@@ -7704,36 +7597,36 @@
       <c r="Y22" s="2"/>
       <c r="Z22" s="2"/>
     </row>
-    <row r="23" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:26" ht="18.75">
       <c r="A23" s="12" t="s">
         <v>92</v>
       </c>
       <c r="B23" s="13"/>
-      <c r="C23" s="136">
+      <c r="C23" s="13">
         <v>6</v>
       </c>
-      <c r="D23" s="136">
+      <c r="D23" s="13">
         <v>7</v>
       </c>
-      <c r="E23" s="136">
-        <v>5</v>
-      </c>
-      <c r="F23" s="136">
+      <c r="E23" s="13">
+        <v>5</v>
+      </c>
+      <c r="F23" s="13">
         <v>6</v>
       </c>
-      <c r="G23" s="136">
-        <v>5</v>
-      </c>
-      <c r="H23" s="136">
+      <c r="G23" s="13">
+        <v>5</v>
+      </c>
+      <c r="H23" s="13">
         <v>7</v>
       </c>
-      <c r="I23" s="136">
-        <v>5</v>
-      </c>
-      <c r="J23" s="136">
-        <v>5</v>
-      </c>
-      <c r="K23" s="136">
+      <c r="I23" s="13">
+        <v>5</v>
+      </c>
+      <c r="J23" s="13">
+        <v>5</v>
+      </c>
+      <c r="K23" s="13">
         <v>6</v>
       </c>
       <c r="L23" s="14">
@@ -7760,7 +7653,7 @@
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
     </row>
-    <row r="24" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="19.5" thickBot="1">
       <c r="A24" s="16"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17">
@@ -7821,7 +7714,7 @@
       <c r="Y24" s="2"/>
       <c r="Z24" s="2"/>
     </row>
-    <row r="25" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26" ht="18.75">
       <c r="A25" s="12" t="s">
         <v>80</v>
       </c>
@@ -7874,7 +7767,7 @@
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
     </row>
-    <row r="26" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="19.5" thickBot="1">
       <c r="A26" s="16"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -7905,7 +7798,7 @@
       <c r="Y26" s="2"/>
       <c r="Z26" s="2"/>
     </row>
-    <row r="27" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:26" ht="18.75">
       <c r="A27" s="12" t="s">
         <v>23</v>
       </c>
@@ -7961,7 +7854,7 @@
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
     </row>
-    <row r="28" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="19.5" thickBot="1">
       <c r="A28" s="16"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17">
@@ -8022,7 +7915,7 @@
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
     </row>
-    <row r="29" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26" ht="18.75">
       <c r="A29" s="12" t="s">
         <v>79</v>
       </c>
@@ -8036,7 +7929,7 @@
       <c r="E29" s="13">
         <v>5</v>
       </c>
-      <c r="F29" s="138">
+      <c r="F29" s="103">
         <v>2</v>
       </c>
       <c r="G29" s="13">
@@ -8078,7 +7971,7 @@
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
     </row>
-    <row r="30" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" ht="19.5" thickBot="1">
       <c r="A30" s="16"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17">
@@ -8139,7 +8032,7 @@
       <c r="Y30" s="2"/>
       <c r="Z30" s="2"/>
     </row>
-    <row r="31" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:26" ht="18.75">
       <c r="A31" s="12" t="s">
         <v>78</v>
       </c>
@@ -8192,7 +8085,7 @@
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
     </row>
-    <row r="32" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" ht="19.5" thickBot="1">
       <c r="A32" s="16"/>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -8226,7 +8119,7 @@
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
     </row>
-    <row r="33" spans="1:26" ht="19" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:26" ht="18.75">
       <c r="A33" s="12" t="s">
         <v>40</v>
       </c>
@@ -8282,7 +8175,7 @@
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
     </row>
-    <row r="34" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" ht="19.5" thickBot="1">
       <c r="A34" s="16"/>
       <c r="B34" s="17"/>
       <c r="C34" s="17">

</xml_diff>